<commit_message>
Cambios paar finalizar el generador base con clases
</commit_message>
<xml_diff>
--- a/data/inputs/reglas_local.xlsx
+++ b/data/inputs/reglas_local.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jaimeteran/Documents/PYTHON/vacanze_romane/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jaimeteran/Documents/PYTHON/VacanzeGIT/data/inputs/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0ADBCD4A-4509-1F40-8080-EAE6BF3233D6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1242FBC5-874B-C94C-9759-AC943F41E36B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="660" windowWidth="29400" windowHeight="17160" xr2:uid="{0CB8002A-4321-7447-B7A9-BC49A85ACC14}"/>
   </bookViews>
@@ -528,5 +528,6 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0"/>
 </worksheet>
 </file>
</xml_diff>